<commit_message>
Assets/data: update (data + supabase)
</commit_message>
<xml_diff>
--- a/word-data/WordList.xlsx
+++ b/word-data/WordList.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miaofang/Desktop/data_prep/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{472929FC-0B1B-9F43-8B60-D3EEB8615A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03B366D3-A95C-884A-B819-2C022A43E1C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1740" yWindow="920" windowWidth="32820" windowHeight="21420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4991" uniqueCount="3708">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5001" uniqueCount="3718">
   <si>
     <t>English</t>
   </si>
@@ -9063,6 +9063,9 @@
     <t>裁判</t>
   </si>
   <si>
+    <t>cáipàn</t>
+  </si>
+  <si>
     <t>主審</t>
   </si>
   <si>
@@ -9096,6 +9099,9 @@
     <t>球迷</t>
   </si>
   <si>
+    <t>qiúmí</t>
+  </si>
+  <si>
     <t>팬</t>
   </si>
   <si>
@@ -9129,6 +9135,9 @@
     <t>球衣</t>
   </si>
   <si>
+    <t>qiúyī</t>
+  </si>
+  <si>
     <t>ユニフォーム</t>
   </si>
   <si>
@@ -9168,6 +9177,9 @@
     <t>草坪</t>
   </si>
   <si>
+    <t>cǎopíng</t>
+  </si>
+  <si>
     <t>芝</t>
   </si>
   <si>
@@ -9204,6 +9216,9 @@
     <t>球门</t>
   </si>
   <si>
+    <t>qiúmén</t>
+  </si>
+  <si>
     <t>ゴール</t>
   </si>
   <si>
@@ -9240,6 +9255,9 @@
     <t>球网</t>
   </si>
   <si>
+    <t>qiúwǎng</t>
+  </si>
+  <si>
     <t>ネット</t>
   </si>
   <si>
@@ -9273,6 +9291,9 @@
     <t>看台</t>
   </si>
   <si>
+    <t>kàntái</t>
+  </si>
+  <si>
     <t>スタンド</t>
   </si>
   <si>
@@ -9309,6 +9330,9 @@
     <t>禁区</t>
   </si>
   <si>
+    <t>jìnqū</t>
+  </si>
+  <si>
     <t>ペナルティーエリア</t>
   </si>
   <si>
@@ -9348,6 +9372,9 @@
     <t>守门员</t>
   </si>
   <si>
+    <t>shǒuményuán</t>
+  </si>
+  <si>
     <t>ゴールキーパー</t>
   </si>
   <si>
@@ -9384,6 +9411,9 @@
     <t>后卫</t>
   </si>
   <si>
+    <t>hòuwèi</t>
+  </si>
+  <si>
     <t>ディフェンダー</t>
   </si>
   <si>
@@ -10692,6 +10722,9 @@
     <t>尼克斯</t>
   </si>
   <si>
+    <t>níkèsī</t>
+  </si>
+  <si>
     <t>尼克斯太爱纽约啦，每场比赛都揣着个小小的自由女神像！</t>
   </si>
   <si>
@@ -11143,9 +11176,6 @@
   </si>
   <si>
     <t>"dark cloud 暗云"是"颜色深"次要义；dark 首要义是"黑暗/无光"</t>
-  </si>
-  <si>
-    <t>níkèsī</t>
   </si>
 </sst>
 </file>
@@ -11677,8 +11707,8 @@
     <col min="18" max="19" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="20" max="21" width="17.5" style="1" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="181" width="8.83203125" style="1" customWidth="1"/>
-    <col min="182" max="16384" width="8.83203125" style="1"/>
+    <col min="23" max="182" width="8.83203125" style="1" customWidth="1"/>
+    <col min="183" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.2">
@@ -24549,8 +24579,8 @@
     <col min="20" max="20" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="21" max="22" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="17.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="27" width="8.83203125" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.83203125" style="1"/>
+    <col min="24" max="28" width="8.83203125" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.2">
@@ -24989,37 +25019,40 @@
       <c r="I10" s="1" t="s">
         <v>3012</v>
       </c>
+      <c r="J10" t="s">
+        <v>3013</v>
+      </c>
       <c r="L10" s="1" t="s">
-        <v>3013</v>
+        <v>3014</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>3014</v>
+        <v>3015</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>3015</v>
+        <v>3016</v>
       </c>
       <c r="R10" s="1" t="s">
+        <v>3017</v>
+      </c>
+      <c r="S10" s="1" t="s">
+        <v>3018</v>
+      </c>
+      <c r="T10" s="1" t="s">
+        <v>3019</v>
+      </c>
+      <c r="U10" s="1" t="s">
         <v>3016</v>
       </c>
-      <c r="S10" s="1" t="s">
-        <v>3017</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>3018</v>
-      </c>
-      <c r="U10" s="1" t="s">
-        <v>3015</v>
-      </c>
       <c r="V10" s="1" t="s">
-        <v>3019</v>
+        <v>3020</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>3020</v>
+        <v>3021</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>3021</v>
+        <v>3022</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>2914</v>
@@ -25028,39 +25061,42 @@
         <v>2915</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>3022</v>
+        <v>3023</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>3023</v>
+        <v>3024</v>
+      </c>
+      <c r="J11" t="s">
+        <v>3025</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>3024</v>
+        <v>3026</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>3025</v>
+        <v>3027</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>3026</v>
+        <v>3028</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>3027</v>
+        <v>3029</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>3028</v>
+        <v>3030</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>3029</v>
+        <v>3031</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>3030</v>
+        <v>3032</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>3031</v>
+        <v>3033</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>3032</v>
+        <v>3034</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>2914</v>
@@ -25069,2414 +25105,2438 @@
         <v>2915</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>3033</v>
+        <v>3035</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>3034</v>
+        <v>3036</v>
+      </c>
+      <c r="J12" t="s">
+        <v>3037</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>3035</v>
+        <v>3038</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>3036</v>
+        <v>3039</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>3037</v>
+        <v>3040</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>3038</v>
+        <v>3041</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>3039</v>
+        <v>3042</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>3040</v>
+        <v>3043</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>3041</v>
+        <v>3044</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>3042</v>
+        <v>3045</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>3043</v>
+        <v>3046</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>3044</v>
+        <v>3047</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>3045</v>
+        <v>3048</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>3046</v>
+        <v>3049</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>3047</v>
+        <v>3050</v>
+      </c>
+      <c r="J13" t="s">
+        <v>3051</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>3048</v>
+        <v>3052</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>3049</v>
+        <v>3053</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>3050</v>
+        <v>3054</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>3051</v>
+        <v>3055</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>3052</v>
+        <v>3056</v>
       </c>
       <c r="T13" s="1" t="s">
-        <v>3053</v>
+        <v>3057</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>3054</v>
+        <v>3058</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>3055</v>
+        <v>3059</v>
       </c>
       <c r="W13" s="1" t="s">
-        <v>3056</v>
+        <v>3060</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>3057</v>
+        <v>3061</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>3045</v>
+        <v>3048</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>3058</v>
+        <v>3062</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>3059</v>
+        <v>3063</v>
+      </c>
+      <c r="J14" t="s">
+        <v>3064</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>3060</v>
+        <v>3065</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>3061</v>
+        <v>3066</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>3062</v>
+        <v>3067</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>3063</v>
+        <v>3068</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>3064</v>
+        <v>3069</v>
       </c>
       <c r="T14" s="1" t="s">
-        <v>3065</v>
+        <v>3070</v>
       </c>
       <c r="U14" s="1" t="s">
-        <v>3066</v>
+        <v>3071</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>3067</v>
+        <v>3072</v>
       </c>
       <c r="W14" s="1" t="s">
-        <v>3068</v>
+        <v>3073</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>3069</v>
+        <v>3074</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>3045</v>
+        <v>3048</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>3070</v>
+        <v>3075</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>3071</v>
+        <v>3076</v>
+      </c>
+      <c r="J15" t="s">
+        <v>3077</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>3072</v>
+        <v>3078</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>3073</v>
+        <v>3079</v>
       </c>
       <c r="Q15" s="1" t="s">
         <v>630</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>3074</v>
+        <v>3080</v>
       </c>
       <c r="S15" s="1" t="s">
-        <v>3075</v>
+        <v>3081</v>
       </c>
       <c r="T15" s="1" t="s">
-        <v>3076</v>
+        <v>3082</v>
       </c>
       <c r="U15" s="1" t="s">
-        <v>3077</v>
+        <v>3083</v>
       </c>
       <c r="V15" s="1" t="s">
-        <v>3078</v>
+        <v>3084</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>3079</v>
+        <v>3085</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>3080</v>
+        <v>3086</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>3045</v>
+        <v>3048</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>3081</v>
+        <v>3087</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>3082</v>
+        <v>3088</v>
+      </c>
+      <c r="J16" t="s">
+        <v>3089</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>3083</v>
+        <v>3090</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>3084</v>
+        <v>3091</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>3085</v>
+        <v>3092</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>3086</v>
+        <v>3093</v>
       </c>
       <c r="S16" s="1" t="s">
-        <v>3087</v>
+        <v>3094</v>
       </c>
       <c r="T16" s="1" t="s">
-        <v>3088</v>
+        <v>3095</v>
       </c>
       <c r="U16" s="1" t="s">
-        <v>3089</v>
+        <v>3096</v>
       </c>
       <c r="V16" s="1" t="s">
-        <v>3090</v>
+        <v>3097</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>3091</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>3092</v>
+        <v>3099</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>3045</v>
+        <v>3048</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>3093</v>
+        <v>3100</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>3094</v>
+        <v>3101</v>
+      </c>
+      <c r="J17" t="s">
+        <v>3102</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>3095</v>
+        <v>3103</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>3096</v>
+        <v>3104</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>3097</v>
+        <v>3105</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>3098</v>
+        <v>3106</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>3099</v>
+        <v>3107</v>
       </c>
       <c r="T17" s="1" t="s">
-        <v>3100</v>
+        <v>3108</v>
       </c>
       <c r="U17" s="1" t="s">
-        <v>3101</v>
+        <v>3109</v>
       </c>
       <c r="V17" s="1" t="s">
-        <v>3102</v>
+        <v>3110</v>
       </c>
       <c r="W17" s="1" t="s">
-        <v>3103</v>
+        <v>3111</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>3104</v>
+        <v>3112</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>3105</v>
+        <v>3113</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>3106</v>
+        <v>3114</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>3107</v>
+        <v>3115</v>
+      </c>
+      <c r="J18" t="s">
+        <v>3116</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>3108</v>
+        <v>3117</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>3109</v>
+        <v>3118</v>
       </c>
       <c r="Q18" s="1" t="s">
-        <v>3110</v>
+        <v>3119</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>3111</v>
+        <v>3120</v>
       </c>
       <c r="S18" s="1" t="s">
-        <v>3112</v>
+        <v>3121</v>
       </c>
       <c r="T18" s="1" t="s">
-        <v>3113</v>
+        <v>3122</v>
       </c>
       <c r="U18" s="1" t="s">
-        <v>3114</v>
+        <v>3123</v>
       </c>
       <c r="V18" s="1" t="s">
-        <v>3115</v>
+        <v>3124</v>
       </c>
       <c r="W18" s="1" t="s">
-        <v>3116</v>
+        <v>3125</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>3117</v>
+        <v>3126</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>3105</v>
+        <v>3113</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>3118</v>
+        <v>3127</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>3119</v>
+        <v>3128</v>
+      </c>
+      <c r="J19" t="s">
+        <v>3129</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>3120</v>
+        <v>3130</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>3121</v>
+        <v>3131</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>3122</v>
+        <v>3132</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>3123</v>
+        <v>3133</v>
       </c>
       <c r="S19" s="1" t="s">
-        <v>3124</v>
+        <v>3134</v>
       </c>
       <c r="T19" s="1" t="s">
-        <v>3125</v>
+        <v>3135</v>
       </c>
       <c r="U19" s="1" t="s">
-        <v>3126</v>
+        <v>3136</v>
       </c>
       <c r="V19" s="1" t="s">
-        <v>3127</v>
+        <v>3137</v>
       </c>
       <c r="W19" s="1" t="s">
-        <v>3128</v>
+        <v>3138</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>3129</v>
+        <v>3139</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>3105</v>
+        <v>3113</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>3130</v>
+        <v>3140</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>3131</v>
+        <v>3141</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>3132</v>
+        <v>3142</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>3133</v>
+        <v>3143</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>3134</v>
+        <v>3144</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>3134</v>
+        <v>3144</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>3135</v>
+        <v>3145</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>3136</v>
+        <v>3146</v>
       </c>
       <c r="U20" s="1" t="s">
-        <v>3137</v>
+        <v>3147</v>
       </c>
       <c r="V20" s="1" t="s">
-        <v>3138</v>
+        <v>3148</v>
       </c>
       <c r="W20" s="1" t="s">
-        <v>3139</v>
+        <v>3149</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>3140</v>
+        <v>3150</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>3105</v>
+        <v>3113</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>3141</v>
+        <v>3151</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>3142</v>
+        <v>3152</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>3143</v>
+        <v>3153</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>3144</v>
+        <v>3154</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>3145</v>
+        <v>3155</v>
       </c>
       <c r="R21" s="1" t="s">
-        <v>3146</v>
+        <v>3156</v>
       </c>
       <c r="S21" s="1" t="s">
-        <v>3147</v>
+        <v>3157</v>
       </c>
       <c r="T21" s="1" t="s">
-        <v>3148</v>
+        <v>3158</v>
       </c>
       <c r="U21" s="1" t="s">
-        <v>3149</v>
+        <v>3159</v>
       </c>
       <c r="V21" s="1" t="s">
-        <v>3150</v>
+        <v>3160</v>
       </c>
       <c r="W21" s="1" t="s">
-        <v>3151</v>
+        <v>3161</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>3152</v>
+        <v>3162</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>3153</v>
+        <v>3163</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>3154</v>
+        <v>3164</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>3155</v>
+        <v>3165</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>3156</v>
+        <v>3166</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>3157</v>
+        <v>3167</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>3158</v>
+        <v>3168</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>3159</v>
+        <v>3169</v>
       </c>
       <c r="S22" s="1" t="s">
-        <v>3160</v>
+        <v>3170</v>
       </c>
       <c r="T22" s="1" t="s">
-        <v>3161</v>
+        <v>3171</v>
       </c>
       <c r="U22" s="1" t="s">
-        <v>3162</v>
+        <v>3172</v>
       </c>
       <c r="V22" s="1" t="s">
-        <v>3163</v>
+        <v>3173</v>
       </c>
       <c r="W22" s="1" t="s">
-        <v>3164</v>
+        <v>3174</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>3165</v>
+        <v>3175</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>3153</v>
+        <v>3163</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>3058</v>
+        <v>3062</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>3166</v>
+        <v>3176</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>3167</v>
+        <v>3177</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>3168</v>
+        <v>3178</v>
       </c>
       <c r="Q23" s="1" t="s">
-        <v>3066</v>
+        <v>3071</v>
       </c>
       <c r="R23" s="1" t="s">
-        <v>3066</v>
+        <v>3071</v>
       </c>
       <c r="S23" s="1" t="s">
-        <v>3064</v>
+        <v>3069</v>
       </c>
       <c r="T23" s="1" t="s">
-        <v>3065</v>
+        <v>3070</v>
       </c>
       <c r="U23" s="1" t="s">
-        <v>3066</v>
+        <v>3071</v>
       </c>
       <c r="V23" s="1" t="s">
-        <v>3169</v>
+        <v>3179</v>
       </c>
       <c r="W23" s="1" t="s">
-        <v>3170</v>
+        <v>3180</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>3171</v>
+        <v>3181</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>3153</v>
+        <v>3163</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>3172</v>
+        <v>3182</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>3173</v>
+        <v>3183</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>3174</v>
+        <v>3184</v>
       </c>
       <c r="P24" s="1" t="s">
-        <v>3175</v>
+        <v>3185</v>
       </c>
       <c r="Q24" s="1" t="s">
-        <v>3176</v>
+        <v>3186</v>
       </c>
       <c r="R24" s="1" t="s">
-        <v>3177</v>
+        <v>3187</v>
       </c>
       <c r="S24" s="1" t="s">
-        <v>3178</v>
+        <v>3188</v>
       </c>
       <c r="T24" s="1" t="s">
-        <v>3179</v>
+        <v>3189</v>
       </c>
       <c r="U24" s="1" t="s">
-        <v>3178</v>
+        <v>3188</v>
       </c>
       <c r="V24" s="1" t="s">
-        <v>3180</v>
+        <v>3190</v>
       </c>
       <c r="W24" s="1" t="s">
-        <v>3181</v>
+        <v>3191</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>3182</v>
+        <v>3192</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>3153</v>
+        <v>3163</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>3183</v>
+        <v>3193</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>3184</v>
+        <v>3194</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>3185</v>
+        <v>3195</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>3186</v>
+        <v>3196</v>
       </c>
       <c r="Q25" s="1" t="s">
-        <v>3187</v>
+        <v>3197</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>3182</v>
+        <v>3192</v>
       </c>
       <c r="S25" s="1" t="s">
-        <v>3188</v>
+        <v>3198</v>
       </c>
       <c r="T25" s="1" t="s">
-        <v>3189</v>
+        <v>3199</v>
       </c>
       <c r="U25" s="1" t="s">
-        <v>3190</v>
+        <v>3200</v>
       </c>
       <c r="V25" s="1" t="s">
-        <v>3191</v>
+        <v>3201</v>
       </c>
       <c r="W25" s="1" t="s">
-        <v>3192</v>
+        <v>3202</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>3193</v>
+        <v>3203</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>3153</v>
+        <v>3163</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>3194</v>
+        <v>3204</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>3195</v>
+        <v>3205</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>3196</v>
+        <v>3206</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>3197</v>
+        <v>3207</v>
       </c>
       <c r="Q26" s="1" t="s">
-        <v>3198</v>
+        <v>3208</v>
       </c>
       <c r="R26" s="1" t="s">
-        <v>3199</v>
+        <v>3209</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>3200</v>
+        <v>3210</v>
       </c>
       <c r="T26" s="1" t="s">
-        <v>3201</v>
+        <v>3211</v>
       </c>
       <c r="U26" s="1" t="s">
-        <v>3198</v>
+        <v>3208</v>
       </c>
       <c r="V26" s="1" t="s">
-        <v>3202</v>
+        <v>3212</v>
       </c>
       <c r="W26" s="1" t="s">
-        <v>3203</v>
+        <v>3213</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>3204</v>
+        <v>3214</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>3153</v>
+        <v>3163</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>3205</v>
+        <v>3215</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>3206</v>
+        <v>3216</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>3207</v>
+        <v>3217</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>3208</v>
+        <v>3218</v>
       </c>
       <c r="Q27" s="1" t="s">
-        <v>3209</v>
+        <v>3219</v>
       </c>
       <c r="R27" s="1" t="s">
-        <v>3209</v>
+        <v>3219</v>
       </c>
       <c r="S27" s="1" t="s">
-        <v>3210</v>
+        <v>3220</v>
       </c>
       <c r="T27" s="1" t="s">
-        <v>3211</v>
+        <v>3221</v>
       </c>
       <c r="U27" s="1" t="s">
-        <v>3212</v>
+        <v>3222</v>
       </c>
       <c r="V27" s="1" t="s">
-        <v>3213</v>
+        <v>3223</v>
       </c>
       <c r="W27" s="1" t="s">
-        <v>3214</v>
+        <v>3224</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>3215</v>
+        <v>3225</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>3153</v>
+        <v>3163</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>3216</v>
+        <v>3226</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>3217</v>
+        <v>3227</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>3218</v>
+        <v>3228</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>3219</v>
+        <v>3229</v>
       </c>
       <c r="Q28" s="1" t="s">
-        <v>3220</v>
+        <v>3230</v>
       </c>
       <c r="R28" s="1" t="s">
-        <v>3221</v>
+        <v>3231</v>
       </c>
       <c r="S28" s="1" t="s">
-        <v>3222</v>
+        <v>3232</v>
       </c>
       <c r="T28" s="1" t="s">
-        <v>3223</v>
+        <v>3233</v>
       </c>
       <c r="U28" s="1" t="s">
-        <v>3224</v>
+        <v>3234</v>
       </c>
       <c r="V28" s="1" t="s">
-        <v>3225</v>
+        <v>3235</v>
       </c>
       <c r="W28" s="1" t="s">
-        <v>3226</v>
+        <v>3236</v>
       </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>3227</v>
+        <v>3237</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>3228</v>
+        <v>3238</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>3229</v>
+        <v>3239</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>3230</v>
+        <v>3240</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>3231</v>
+        <v>3241</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>3232</v>
+        <v>3242</v>
       </c>
       <c r="Q29" s="1" t="s">
-        <v>3233</v>
+        <v>3243</v>
       </c>
       <c r="R29" s="1" t="s">
-        <v>3234</v>
+        <v>3244</v>
       </c>
       <c r="S29" s="1" t="s">
-        <v>3235</v>
+        <v>3245</v>
       </c>
       <c r="T29" s="1" t="s">
-        <v>3236</v>
+        <v>3246</v>
       </c>
       <c r="U29" s="1" t="s">
-        <v>3237</v>
+        <v>3247</v>
       </c>
       <c r="V29" s="1" t="s">
-        <v>3238</v>
+        <v>3248</v>
       </c>
       <c r="W29" s="1" t="s">
-        <v>3239</v>
+        <v>3249</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>3240</v>
+        <v>3250</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>3228</v>
+        <v>3238</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>3241</v>
+        <v>3251</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>3242</v>
+        <v>3252</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>3243</v>
+        <v>3253</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>3244</v>
+        <v>3254</v>
       </c>
       <c r="Q30" s="1" t="s">
-        <v>3245</v>
+        <v>3255</v>
       </c>
       <c r="R30" s="1" t="s">
-        <v>3246</v>
+        <v>3256</v>
       </c>
       <c r="S30" s="1" t="s">
-        <v>3240</v>
+        <v>3250</v>
       </c>
       <c r="T30" s="1" t="s">
-        <v>3247</v>
+        <v>3257</v>
       </c>
       <c r="U30" s="1" t="s">
-        <v>3248</v>
+        <v>3258</v>
       </c>
       <c r="V30" s="1" t="s">
-        <v>3249</v>
+        <v>3259</v>
       </c>
       <c r="W30" s="1" t="s">
-        <v>3250</v>
+        <v>3260</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>3251</v>
+        <v>3261</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>3228</v>
+        <v>3238</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>3252</v>
+        <v>3262</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>3253</v>
+        <v>3263</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>3254</v>
+        <v>3264</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>3255</v>
+        <v>3265</v>
       </c>
       <c r="Q31" s="1" t="s">
-        <v>3256</v>
+        <v>3266</v>
       </c>
       <c r="R31" s="1" t="s">
-        <v>3257</v>
+        <v>3267</v>
       </c>
       <c r="S31" s="1" t="s">
-        <v>3258</v>
+        <v>3268</v>
       </c>
       <c r="T31" s="1" t="s">
-        <v>3259</v>
+        <v>3269</v>
       </c>
       <c r="U31" s="1" t="s">
-        <v>3260</v>
+        <v>3270</v>
       </c>
       <c r="V31" s="1" t="s">
-        <v>3261</v>
+        <v>3271</v>
       </c>
       <c r="W31" s="1" t="s">
-        <v>3262</v>
+        <v>3272</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>3263</v>
+        <v>3273</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>3228</v>
+        <v>3238</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>3264</v>
+        <v>3274</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>3265</v>
+        <v>3275</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>3266</v>
+        <v>3276</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>3267</v>
+        <v>3277</v>
       </c>
       <c r="Q32" s="1" t="s">
-        <v>3268</v>
+        <v>3278</v>
       </c>
       <c r="R32" s="1" t="s">
-        <v>3269</v>
+        <v>3279</v>
       </c>
       <c r="S32" s="1" t="s">
-        <v>3270</v>
+        <v>3280</v>
       </c>
       <c r="T32" s="1" t="s">
-        <v>3271</v>
+        <v>3281</v>
       </c>
       <c r="U32" s="1" t="s">
-        <v>3272</v>
+        <v>3282</v>
       </c>
       <c r="V32" s="1" t="s">
-        <v>3273</v>
+        <v>3283</v>
       </c>
       <c r="W32" s="1" t="s">
-        <v>3274</v>
+        <v>3284</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>3275</v>
+        <v>3285</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>3228</v>
+        <v>3238</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>3276</v>
+        <v>3286</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>3277</v>
+        <v>3287</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>3278</v>
+        <v>3288</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>3279</v>
+        <v>3289</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>3280</v>
+        <v>3290</v>
       </c>
       <c r="R33" s="1" t="s">
-        <v>3281</v>
+        <v>3291</v>
       </c>
       <c r="S33" s="1" t="s">
-        <v>3282</v>
+        <v>3292</v>
       </c>
       <c r="T33" s="1" t="s">
-        <v>3283</v>
+        <v>3293</v>
       </c>
       <c r="U33" s="1" t="s">
-        <v>3284</v>
+        <v>3294</v>
       </c>
       <c r="V33" s="1" t="s">
-        <v>3285</v>
+        <v>3295</v>
       </c>
       <c r="W33" s="1" t="s">
-        <v>3286</v>
+        <v>3296</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>3287</v>
+        <v>3297</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>3228</v>
+        <v>3238</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>3288</v>
+        <v>3298</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>3289</v>
+        <v>3299</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>3290</v>
+        <v>3300</v>
       </c>
       <c r="P34" s="1" t="s">
-        <v>3291</v>
+        <v>3301</v>
       </c>
       <c r="Q34" s="1" t="s">
-        <v>3292</v>
+        <v>3302</v>
       </c>
       <c r="R34" s="1" t="s">
-        <v>3293</v>
+        <v>3303</v>
       </c>
       <c r="S34" s="1" t="s">
-        <v>3294</v>
+        <v>3304</v>
       </c>
       <c r="T34" s="1" t="s">
-        <v>3295</v>
+        <v>3305</v>
       </c>
       <c r="U34" s="1" t="s">
-        <v>3296</v>
+        <v>3306</v>
       </c>
       <c r="V34" s="1" t="s">
-        <v>3297</v>
+        <v>3307</v>
       </c>
       <c r="W34" s="1" t="s">
-        <v>3298</v>
+        <v>3308</v>
       </c>
     </row>
     <row r="35" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>3299</v>
+        <v>3309</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>3228</v>
+        <v>3238</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>3300</v>
+        <v>3310</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>3301</v>
+        <v>3311</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>3302</v>
+        <v>3312</v>
       </c>
       <c r="P35" s="1" t="s">
-        <v>3303</v>
+        <v>3313</v>
       </c>
       <c r="Q35" s="1" t="s">
-        <v>3304</v>
+        <v>3314</v>
       </c>
       <c r="R35" s="1" t="s">
-        <v>3305</v>
+        <v>3315</v>
       </c>
       <c r="S35" s="1" t="s">
-        <v>3306</v>
+        <v>3316</v>
       </c>
       <c r="T35" s="1" t="s">
-        <v>3307</v>
+        <v>3317</v>
       </c>
       <c r="U35" s="1" t="s">
-        <v>3308</v>
+        <v>3318</v>
       </c>
       <c r="V35" s="1" t="s">
-        <v>3309</v>
+        <v>3319</v>
       </c>
       <c r="W35" s="1" t="s">
-        <v>3310</v>
+        <v>3320</v>
       </c>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>3311</v>
+        <v>3321</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>3313</v>
+        <v>3323</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>3314</v>
+        <v>3324</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>3315</v>
+        <v>3325</v>
       </c>
       <c r="P36" s="1" t="s">
-        <v>3316</v>
+        <v>3326</v>
       </c>
       <c r="Q36" s="1" t="s">
-        <v>3317</v>
+        <v>3327</v>
       </c>
       <c r="R36" s="1" t="s">
-        <v>3318</v>
+        <v>3328</v>
       </c>
       <c r="S36" s="1" t="s">
-        <v>3319</v>
+        <v>3329</v>
       </c>
       <c r="T36" s="1" t="s">
-        <v>3320</v>
+        <v>3330</v>
       </c>
       <c r="U36" s="1" t="s">
-        <v>3317</v>
+        <v>3327</v>
       </c>
       <c r="V36" s="1" t="s">
-        <v>3321</v>
+        <v>3331</v>
       </c>
       <c r="W36" s="1" t="s">
-        <v>3322</v>
+        <v>3332</v>
       </c>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>3323</v>
+        <v>3333</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>3324</v>
+        <v>3334</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>3325</v>
+        <v>3335</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>3326</v>
+        <v>3336</v>
       </c>
       <c r="P37" s="1" t="s">
-        <v>3327</v>
+        <v>3337</v>
       </c>
       <c r="Q37" s="1" t="s">
-        <v>3328</v>
+        <v>3338</v>
       </c>
       <c r="R37" s="1" t="s">
-        <v>3329</v>
+        <v>3339</v>
       </c>
       <c r="S37" s="1" t="s">
-        <v>3330</v>
+        <v>3340</v>
       </c>
       <c r="T37" s="1" t="s">
-        <v>3331</v>
+        <v>3341</v>
       </c>
       <c r="U37" s="1" t="s">
-        <v>3332</v>
+        <v>3342</v>
       </c>
       <c r="V37" s="1" t="s">
-        <v>3333</v>
+        <v>3343</v>
       </c>
       <c r="W37" s="1" t="s">
-        <v>3334</v>
+        <v>3344</v>
       </c>
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>3335</v>
+        <v>3345</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>3336</v>
+        <v>3346</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>3337</v>
+        <v>3347</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>3338</v>
+        <v>3348</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>3339</v>
+        <v>3349</v>
       </c>
       <c r="Q38" s="1" t="s">
-        <v>3340</v>
+        <v>3350</v>
       </c>
       <c r="R38" s="1" t="s">
-        <v>3341</v>
+        <v>3351</v>
       </c>
       <c r="S38" s="1" t="s">
-        <v>3342</v>
+        <v>3352</v>
       </c>
       <c r="T38" s="1" t="s">
-        <v>3343</v>
+        <v>3353</v>
       </c>
       <c r="U38" s="1" t="s">
-        <v>3344</v>
+        <v>3354</v>
       </c>
       <c r="V38" s="1" t="s">
-        <v>3345</v>
+        <v>3355</v>
       </c>
       <c r="W38" s="1" t="s">
-        <v>3346</v>
+        <v>3356</v>
       </c>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>3347</v>
+        <v>3357</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>3348</v>
+        <v>3358</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>3349</v>
+        <v>3359</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>3350</v>
+        <v>3360</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>3351</v>
+        <v>3361</v>
       </c>
       <c r="Q39" s="1" t="s">
-        <v>3352</v>
+        <v>3362</v>
       </c>
       <c r="R39" s="1" t="s">
-        <v>3353</v>
+        <v>3363</v>
       </c>
       <c r="S39" s="1" t="s">
-        <v>3354</v>
+        <v>3364</v>
       </c>
       <c r="T39" s="1" t="s">
-        <v>3355</v>
+        <v>3365</v>
       </c>
       <c r="U39" s="1" t="s">
-        <v>3356</v>
+        <v>3366</v>
       </c>
       <c r="V39" s="1" t="s">
-        <v>3357</v>
+        <v>3367</v>
       </c>
       <c r="W39" s="1" t="s">
-        <v>3358</v>
+        <v>3368</v>
       </c>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>3359</v>
+        <v>3369</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>3360</v>
+        <v>3370</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>3361</v>
+        <v>3371</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>3362</v>
+        <v>3372</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>3363</v>
+        <v>3373</v>
       </c>
       <c r="Q40" s="1" t="s">
-        <v>3359</v>
+        <v>3369</v>
       </c>
       <c r="R40" s="1" t="s">
-        <v>3364</v>
+        <v>3374</v>
       </c>
       <c r="S40" s="1" t="s">
-        <v>3365</v>
+        <v>3375</v>
       </c>
       <c r="T40" s="1" t="s">
-        <v>3366</v>
+        <v>3376</v>
       </c>
       <c r="U40" s="1" t="s">
-        <v>3359</v>
+        <v>3369</v>
       </c>
       <c r="V40" s="1" t="s">
-        <v>3367</v>
+        <v>3377</v>
       </c>
       <c r="W40" s="1" t="s">
-        <v>3368</v>
+        <v>3378</v>
       </c>
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>3369</v>
+        <v>3379</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>3370</v>
+        <v>3380</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>3371</v>
+        <v>3381</v>
       </c>
       <c r="L41" s="1" t="s">
-        <v>3372</v>
+        <v>3382</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>3373</v>
+        <v>3383</v>
       </c>
       <c r="Q41" s="1" t="s">
-        <v>3369</v>
+        <v>3379</v>
       </c>
       <c r="R41" s="1" t="s">
-        <v>3374</v>
+        <v>3384</v>
       </c>
       <c r="S41" s="1" t="s">
-        <v>3374</v>
+        <v>3384</v>
       </c>
       <c r="T41" s="1" t="s">
-        <v>3375</v>
+        <v>3385</v>
       </c>
       <c r="U41" s="1" t="s">
-        <v>3369</v>
+        <v>3379</v>
       </c>
       <c r="V41" s="1" t="s">
-        <v>3376</v>
+        <v>3386</v>
       </c>
       <c r="W41" s="1" t="s">
-        <v>3377</v>
+        <v>3387</v>
       </c>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>3378</v>
+        <v>3388</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>3379</v>
+        <v>3389</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>3380</v>
+        <v>3390</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>3381</v>
+        <v>3391</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>3382</v>
+        <v>3392</v>
       </c>
       <c r="Q42" s="1" t="s">
-        <v>3383</v>
+        <v>3393</v>
       </c>
       <c r="R42" s="1" t="s">
-        <v>3384</v>
+        <v>3394</v>
       </c>
       <c r="S42" s="1" t="s">
-        <v>3385</v>
+        <v>3395</v>
       </c>
       <c r="T42" s="1" t="s">
-        <v>3386</v>
+        <v>3396</v>
       </c>
       <c r="U42" s="1" t="s">
-        <v>3387</v>
+        <v>3397</v>
       </c>
       <c r="V42" s="1" t="s">
-        <v>3388</v>
+        <v>3398</v>
       </c>
       <c r="W42" s="1" t="s">
-        <v>3389</v>
+        <v>3399</v>
       </c>
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>3390</v>
+        <v>3400</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>3391</v>
+        <v>3401</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>3392</v>
+        <v>3402</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>3393</v>
+        <v>3403</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>3394</v>
+        <v>3404</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>3395</v>
+        <v>3405</v>
       </c>
       <c r="R43" s="1" t="s">
-        <v>3396</v>
+        <v>3406</v>
       </c>
       <c r="S43" s="1" t="s">
-        <v>3397</v>
+        <v>3407</v>
       </c>
       <c r="T43" s="1" t="s">
-        <v>3398</v>
+        <v>3408</v>
       </c>
       <c r="U43" s="1" t="s">
-        <v>3399</v>
+        <v>3409</v>
       </c>
       <c r="V43" s="1" t="s">
-        <v>3400</v>
+        <v>3410</v>
       </c>
       <c r="W43" s="1" t="s">
-        <v>3401</v>
+        <v>3411</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>3402</v>
+        <v>3412</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>3403</v>
+        <v>3413</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>3404</v>
+        <v>3414</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>3405</v>
+        <v>3415</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>3406</v>
+        <v>3416</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>3407</v>
+        <v>3417</v>
       </c>
       <c r="R44" s="1" t="s">
-        <v>3408</v>
+        <v>3418</v>
       </c>
       <c r="S44" s="1" t="s">
-        <v>3402</v>
+        <v>3412</v>
       </c>
       <c r="T44" s="1" t="s">
-        <v>3409</v>
+        <v>3419</v>
       </c>
       <c r="U44" s="1" t="s">
-        <v>3410</v>
+        <v>3420</v>
       </c>
       <c r="V44" s="1" t="s">
-        <v>3411</v>
+        <v>3421</v>
       </c>
       <c r="W44" s="1" t="s">
-        <v>3412</v>
+        <v>3422</v>
       </c>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>3413</v>
+        <v>3423</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>3414</v>
+        <v>3424</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>3415</v>
+        <v>3425</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>3416</v>
+        <v>3426</v>
       </c>
       <c r="P45" s="1" t="s">
-        <v>3417</v>
+        <v>3427</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>3418</v>
+        <v>3428</v>
       </c>
       <c r="R45" s="1" t="s">
-        <v>3419</v>
+        <v>3429</v>
       </c>
       <c r="S45" s="1" t="s">
-        <v>3420</v>
+        <v>3430</v>
       </c>
       <c r="T45" s="1" t="s">
-        <v>3421</v>
+        <v>3431</v>
       </c>
       <c r="U45" s="1" t="s">
-        <v>3422</v>
+        <v>3432</v>
       </c>
       <c r="V45" s="1" t="s">
-        <v>3423</v>
+        <v>3433</v>
       </c>
       <c r="W45" s="1" t="s">
-        <v>3424</v>
+        <v>3434</v>
       </c>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>3425</v>
+        <v>3435</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>3312</v>
+        <v>3322</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>3426</v>
+        <v>3436</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>3427</v>
+        <v>3437</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>3428</v>
+        <v>3438</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>3429</v>
+        <v>3439</v>
       </c>
       <c r="Q46" s="1" t="s">
-        <v>3430</v>
+        <v>3440</v>
       </c>
       <c r="R46" s="1" t="s">
-        <v>3431</v>
+        <v>3441</v>
       </c>
       <c r="S46" s="1" t="s">
-        <v>3432</v>
+        <v>3442</v>
       </c>
       <c r="T46" s="1" t="s">
-        <v>3433</v>
+        <v>3443</v>
       </c>
       <c r="U46" s="1" t="s">
-        <v>3434</v>
+        <v>3444</v>
       </c>
       <c r="V46" s="1" t="s">
-        <v>3435</v>
+        <v>3445</v>
       </c>
       <c r="W46" s="1" t="s">
-        <v>3436</v>
+        <v>3446</v>
       </c>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>3437</v>
+        <v>3447</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>3438</v>
+        <v>3448</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>3439</v>
+        <v>3449</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>3440</v>
+        <v>3450</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>3441</v>
+        <v>3451</v>
       </c>
       <c r="P47" s="1" t="s">
-        <v>3442</v>
+        <v>3452</v>
       </c>
       <c r="Q47" s="1" t="s">
-        <v>3437</v>
+        <v>3447</v>
       </c>
       <c r="R47" s="1" t="s">
-        <v>3437</v>
+        <v>3447</v>
       </c>
       <c r="S47" s="1" t="s">
-        <v>3437</v>
+        <v>3447</v>
       </c>
       <c r="T47" s="1" t="s">
-        <v>3437</v>
+        <v>3447</v>
       </c>
       <c r="U47" s="1" t="s">
-        <v>3437</v>
+        <v>3447</v>
       </c>
       <c r="V47" s="1" t="s">
-        <v>3443</v>
+        <v>3453</v>
       </c>
       <c r="W47" s="1" t="s">
-        <v>3444</v>
+        <v>3454</v>
       </c>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>3445</v>
+        <v>3455</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>3438</v>
+        <v>3448</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>3446</v>
+        <v>3456</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>3447</v>
+        <v>3457</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>3448</v>
+        <v>3458</v>
       </c>
       <c r="P48" s="1" t="s">
-        <v>3449</v>
+        <v>3459</v>
       </c>
       <c r="Q48" s="1" t="s">
-        <v>3445</v>
+        <v>3455</v>
       </c>
       <c r="R48" s="1" t="s">
-        <v>3445</v>
+        <v>3455</v>
       </c>
       <c r="S48" s="1" t="s">
-        <v>3445</v>
+        <v>3455</v>
       </c>
       <c r="T48" s="1" t="s">
-        <v>3445</v>
+        <v>3455</v>
       </c>
       <c r="U48" s="1" t="s">
-        <v>3445</v>
+        <v>3455</v>
       </c>
       <c r="V48" s="1" t="s">
-        <v>3450</v>
+        <v>3460</v>
       </c>
       <c r="W48" s="1" t="s">
-        <v>3451</v>
+        <v>3461</v>
       </c>
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>3452</v>
+        <v>3462</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>3438</v>
+        <v>3448</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>3453</v>
+        <v>3463</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>3454</v>
+        <v>3464</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>3455</v>
+        <v>3465</v>
       </c>
       <c r="P49" s="1" t="s">
-        <v>3456</v>
+        <v>3466</v>
       </c>
       <c r="Q49" s="1" t="s">
-        <v>3452</v>
+        <v>3462</v>
       </c>
       <c r="R49" s="1" t="s">
-        <v>3452</v>
+        <v>3462</v>
       </c>
       <c r="S49" s="1" t="s">
-        <v>3452</v>
+        <v>3462</v>
       </c>
       <c r="T49" s="1" t="s">
-        <v>3452</v>
+        <v>3462</v>
       </c>
       <c r="U49" s="1" t="s">
-        <v>3452</v>
+        <v>3462</v>
       </c>
       <c r="V49" s="1" t="s">
-        <v>3457</v>
+        <v>3467</v>
       </c>
       <c r="W49" s="1" t="s">
-        <v>3458</v>
+        <v>3468</v>
       </c>
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>3459</v>
+        <v>3469</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>3438</v>
+        <v>3448</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>3460</v>
+        <v>3470</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>3461</v>
+        <v>3471</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>3462</v>
+        <v>3472</v>
       </c>
       <c r="P50" s="1" t="s">
-        <v>3463</v>
+        <v>3473</v>
       </c>
       <c r="Q50" s="1" t="s">
-        <v>3459</v>
+        <v>3469</v>
       </c>
       <c r="R50" s="1" t="s">
-        <v>3459</v>
+        <v>3469</v>
       </c>
       <c r="S50" s="1" t="s">
-        <v>3459</v>
+        <v>3469</v>
       </c>
       <c r="T50" s="1" t="s">
-        <v>3459</v>
+        <v>3469</v>
       </c>
       <c r="U50" s="1" t="s">
-        <v>3459</v>
+        <v>3469</v>
       </c>
       <c r="V50" s="1" t="s">
-        <v>3464</v>
+        <v>3474</v>
       </c>
       <c r="W50" s="1" t="s">
-        <v>3465</v>
+        <v>3475</v>
       </c>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>3466</v>
+        <v>3476</v>
       </c>
       <c r="F51" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>3438</v>
+        <v>3448</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>3467</v>
+        <v>3477</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>3468</v>
+        <v>3478</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>3469</v>
+        <v>3479</v>
       </c>
       <c r="P51" s="1" t="s">
-        <v>3470</v>
+        <v>3480</v>
       </c>
       <c r="Q51" s="1" t="s">
-        <v>3466</v>
+        <v>3476</v>
       </c>
       <c r="R51" s="1" t="s">
-        <v>3466</v>
+        <v>3476</v>
       </c>
       <c r="S51" s="1" t="s">
-        <v>3466</v>
+        <v>3476</v>
       </c>
       <c r="T51" s="1" t="s">
-        <v>3466</v>
+        <v>3476</v>
       </c>
       <c r="U51" s="1" t="s">
-        <v>3466</v>
+        <v>3476</v>
       </c>
       <c r="V51" s="1" t="s">
-        <v>3471</v>
+        <v>3481</v>
       </c>
       <c r="W51" s="1" t="s">
-        <v>3472</v>
+        <v>3482</v>
       </c>
     </row>
     <row r="52" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>3473</v>
+        <v>3483</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>3438</v>
+        <v>3448</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>3474</v>
+        <v>3484</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>3475</v>
+        <v>3485</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>3476</v>
+        <v>3486</v>
       </c>
       <c r="P52" s="1" t="s">
-        <v>3477</v>
+        <v>3487</v>
       </c>
       <c r="Q52" s="1" t="s">
-        <v>3473</v>
+        <v>3483</v>
       </c>
       <c r="R52" s="1" t="s">
-        <v>3473</v>
+        <v>3483</v>
       </c>
       <c r="S52" s="1" t="s">
-        <v>3473</v>
+        <v>3483</v>
       </c>
       <c r="T52" s="1" t="s">
-        <v>3473</v>
+        <v>3483</v>
       </c>
       <c r="U52" s="1" t="s">
-        <v>3473</v>
+        <v>3483</v>
       </c>
       <c r="V52" s="1" t="s">
-        <v>3478</v>
+        <v>3488</v>
       </c>
       <c r="W52" s="1" t="s">
-        <v>3479</v>
+        <v>3489</v>
       </c>
     </row>
     <row r="53" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>3480</v>
+        <v>3490</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>3438</v>
+        <v>3448</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>3481</v>
+        <v>3491</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>3482</v>
+        <v>3492</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>3483</v>
+        <v>3493</v>
       </c>
       <c r="P53" s="1" t="s">
-        <v>3484</v>
+        <v>3494</v>
       </c>
       <c r="Q53" s="1" t="s">
-        <v>3480</v>
+        <v>3490</v>
       </c>
       <c r="R53" s="1" t="s">
-        <v>3480</v>
+        <v>3490</v>
       </c>
       <c r="S53" s="1" t="s">
-        <v>3480</v>
+        <v>3490</v>
       </c>
       <c r="T53" s="1" t="s">
-        <v>3480</v>
+        <v>3490</v>
       </c>
       <c r="U53" s="1" t="s">
-        <v>3480</v>
+        <v>3490</v>
       </c>
       <c r="V53" s="1" t="s">
-        <v>3485</v>
+        <v>3495</v>
       </c>
       <c r="W53" s="1" t="s">
-        <v>3486</v>
+        <v>3496</v>
       </c>
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>3487</v>
+        <v>3497</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>3438</v>
+        <v>3448</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>3488</v>
+        <v>3498</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>3489</v>
+        <v>3499</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>3490</v>
+        <v>3500</v>
       </c>
       <c r="P54" s="1" t="s">
-        <v>3491</v>
+        <v>3501</v>
       </c>
       <c r="Q54" s="1" t="s">
-        <v>3487</v>
+        <v>3497</v>
       </c>
       <c r="R54" s="1" t="s">
-        <v>3487</v>
+        <v>3497</v>
       </c>
       <c r="S54" s="1" t="s">
-        <v>3487</v>
+        <v>3497</v>
       </c>
       <c r="T54" s="1" t="s">
-        <v>3487</v>
+        <v>3497</v>
       </c>
       <c r="U54" s="1" t="s">
-        <v>3487</v>
+        <v>3497</v>
       </c>
       <c r="V54" s="1" t="s">
-        <v>3492</v>
+        <v>3502</v>
       </c>
       <c r="W54" s="1" t="s">
-        <v>3493</v>
+        <v>3503</v>
       </c>
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>3494</v>
+        <v>3504</v>
       </c>
       <c r="F55" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>3495</v>
+        <v>3505</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>3496</v>
+        <v>3506</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>3497</v>
+        <v>3507</v>
       </c>
       <c r="L55" s="1" t="s">
-        <v>3498</v>
+        <v>3508</v>
       </c>
       <c r="P55" s="1" t="s">
-        <v>3499</v>
+        <v>3509</v>
       </c>
       <c r="Q55" s="1" t="s">
-        <v>3494</v>
+        <v>3504</v>
       </c>
       <c r="R55" s="1" t="s">
-        <v>3494</v>
+        <v>3504</v>
       </c>
       <c r="S55" s="1" t="s">
-        <v>3494</v>
+        <v>3504</v>
       </c>
       <c r="T55" s="1" t="s">
-        <v>3494</v>
+        <v>3504</v>
       </c>
       <c r="U55" s="1" t="s">
-        <v>3494</v>
+        <v>3504</v>
       </c>
       <c r="V55" s="1" t="s">
-        <v>3500</v>
+        <v>3510</v>
       </c>
       <c r="W55" s="1" t="s">
-        <v>3501</v>
+        <v>3511</v>
       </c>
     </row>
     <row r="56" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>3502</v>
+        <v>3512</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>3495</v>
+        <v>3505</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>3503</v>
+        <v>3513</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>3504</v>
+        <v>3514</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>3505</v>
+        <v>3515</v>
       </c>
       <c r="P56" s="1" t="s">
-        <v>3506</v>
+        <v>3516</v>
       </c>
       <c r="Q56" s="1" t="s">
-        <v>3502</v>
+        <v>3512</v>
       </c>
       <c r="R56" s="1" t="s">
-        <v>3502</v>
+        <v>3512</v>
       </c>
       <c r="S56" s="1" t="s">
-        <v>3502</v>
+        <v>3512</v>
       </c>
       <c r="T56" s="1" t="s">
-        <v>3502</v>
+        <v>3512</v>
       </c>
       <c r="U56" s="1" t="s">
-        <v>3502</v>
+        <v>3512</v>
       </c>
       <c r="V56" s="1" t="s">
-        <v>3507</v>
+        <v>3517</v>
       </c>
       <c r="W56" s="1" t="s">
-        <v>3508</v>
+        <v>3518</v>
       </c>
     </row>
     <row r="57" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>3509</v>
+        <v>3519</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>3495</v>
+        <v>3505</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>3510</v>
+        <v>3520</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>3511</v>
+        <v>3521</v>
       </c>
       <c r="L57" s="1" t="s">
-        <v>3512</v>
+        <v>3522</v>
       </c>
       <c r="P57" s="1" t="s">
-        <v>3513</v>
+        <v>3523</v>
       </c>
       <c r="Q57" s="1" t="s">
-        <v>3509</v>
+        <v>3519</v>
       </c>
       <c r="R57" s="1" t="s">
-        <v>3509</v>
+        <v>3519</v>
       </c>
       <c r="S57" s="1" t="s">
-        <v>3509</v>
+        <v>3519</v>
       </c>
       <c r="T57" s="1" t="s">
-        <v>3509</v>
+        <v>3519</v>
       </c>
       <c r="U57" s="1" t="s">
-        <v>3509</v>
+        <v>3519</v>
       </c>
       <c r="V57" s="1" t="s">
-        <v>3514</v>
+        <v>3524</v>
       </c>
       <c r="W57" s="1" t="s">
-        <v>3515</v>
+        <v>3525</v>
       </c>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>3516</v>
+        <v>3526</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>3495</v>
+        <v>3505</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>3517</v>
+        <v>3527</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>3518</v>
+        <v>3528</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>3519</v>
+        <v>3529</v>
       </c>
       <c r="P58" s="1" t="s">
-        <v>3520</v>
+        <v>3530</v>
       </c>
       <c r="Q58" s="1" t="s">
-        <v>3516</v>
+        <v>3526</v>
       </c>
       <c r="R58" s="1" t="s">
-        <v>3516</v>
+        <v>3526</v>
       </c>
       <c r="S58" s="1" t="s">
-        <v>3516</v>
+        <v>3526</v>
       </c>
       <c r="T58" s="1" t="s">
-        <v>3516</v>
+        <v>3526</v>
       </c>
       <c r="U58" s="1" t="s">
-        <v>3516</v>
+        <v>3526</v>
       </c>
       <c r="V58" s="1" t="s">
-        <v>3521</v>
+        <v>3531</v>
       </c>
       <c r="W58" s="1" t="s">
-        <v>3522</v>
+        <v>3532</v>
       </c>
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>3523</v>
+        <v>3533</v>
       </c>
       <c r="F59" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>3495</v>
+        <v>3505</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>3524</v>
+        <v>3534</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>3525</v>
+        <v>3535</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>3526</v>
+        <v>3536</v>
       </c>
       <c r="P59" s="1" t="s">
-        <v>3527</v>
+        <v>3537</v>
       </c>
       <c r="Q59" s="1" t="s">
-        <v>3523</v>
+        <v>3533</v>
       </c>
       <c r="R59" s="1" t="s">
-        <v>3523</v>
+        <v>3533</v>
       </c>
       <c r="S59" s="1" t="s">
-        <v>3523</v>
+        <v>3533</v>
       </c>
       <c r="T59" s="1" t="s">
-        <v>3523</v>
+        <v>3533</v>
       </c>
       <c r="U59" s="1" t="s">
-        <v>3523</v>
+        <v>3533</v>
       </c>
       <c r="V59" s="1" t="s">
-        <v>3528</v>
+        <v>3538</v>
       </c>
       <c r="W59" s="1" t="s">
-        <v>3529</v>
+        <v>3539</v>
       </c>
     </row>
     <row r="60" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>3530</v>
+        <v>3540</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>3495</v>
+        <v>3505</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>3503</v>
+        <v>3513</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>3531</v>
+        <v>3541</v>
       </c>
       <c r="L60" s="1" t="s">
-        <v>3532</v>
+        <v>3542</v>
       </c>
       <c r="P60" s="1" t="s">
-        <v>3533</v>
+        <v>3543</v>
       </c>
       <c r="Q60" s="1" t="s">
-        <v>3530</v>
+        <v>3540</v>
       </c>
       <c r="R60" s="1" t="s">
-        <v>3530</v>
+        <v>3540</v>
       </c>
       <c r="S60" s="1" t="s">
-        <v>3530</v>
+        <v>3540</v>
       </c>
       <c r="T60" s="1" t="s">
-        <v>3530</v>
+        <v>3540</v>
       </c>
       <c r="U60" s="1" t="s">
-        <v>3530</v>
+        <v>3540</v>
       </c>
       <c r="V60" s="1" t="s">
-        <v>3534</v>
+        <v>3544</v>
       </c>
       <c r="W60" s="1" t="s">
-        <v>3535</v>
+        <v>3545</v>
       </c>
     </row>
     <row r="61" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>3536</v>
+        <v>3546</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>3495</v>
+        <v>3505</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>3537</v>
+        <v>3547</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>3538</v>
+        <v>3548</v>
       </c>
       <c r="L61" s="1" t="s">
-        <v>3539</v>
+        <v>3549</v>
       </c>
       <c r="P61" s="1" t="s">
-        <v>3540</v>
+        <v>3550</v>
       </c>
       <c r="Q61" s="1" t="s">
-        <v>3536</v>
+        <v>3546</v>
       </c>
       <c r="R61" s="1" t="s">
-        <v>3536</v>
+        <v>3546</v>
       </c>
       <c r="S61" s="1" t="s">
-        <v>3536</v>
+        <v>3546</v>
       </c>
       <c r="T61" s="1" t="s">
-        <v>3536</v>
+        <v>3546</v>
       </c>
       <c r="U61" s="1" t="s">
-        <v>3536</v>
+        <v>3546</v>
       </c>
       <c r="V61" s="1" t="s">
-        <v>3541</v>
+        <v>3551</v>
       </c>
       <c r="W61" s="1" t="s">
-        <v>3542</v>
+        <v>3552</v>
       </c>
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>3543</v>
+        <v>3553</v>
       </c>
       <c r="F62" s="1" t="s">
         <v>2914</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>3495</v>
+        <v>3505</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>3544</v>
+        <v>3554</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>3545</v>
+        <v>3555</v>
       </c>
       <c r="L62" s="1" t="s">
-        <v>3546</v>
+        <v>3556</v>
       </c>
       <c r="P62" s="1" t="s">
-        <v>3547</v>
+        <v>3557</v>
       </c>
       <c r="Q62" s="1" t="s">
-        <v>3543</v>
+        <v>3553</v>
       </c>
       <c r="R62" s="1" t="s">
-        <v>3543</v>
+        <v>3553</v>
       </c>
       <c r="S62" s="1" t="s">
-        <v>3543</v>
+        <v>3553</v>
       </c>
       <c r="T62" s="1" t="s">
-        <v>3543</v>
+        <v>3553</v>
       </c>
       <c r="U62" s="1" t="s">
-        <v>3543</v>
+        <v>3553</v>
       </c>
       <c r="V62" s="1" t="s">
-        <v>3548</v>
+        <v>3558</v>
       </c>
       <c r="W62" s="1" t="s">
-        <v>3549</v>
+        <v>3559</v>
       </c>
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>3550</v>
+        <v>3560</v>
       </c>
       <c r="C63" t="s">
-        <v>3551</v>
+        <v>3561</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>3552</v>
+        <v>3562</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>3553</v>
+        <v>3563</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>3554</v>
+        <v>3564</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>3555</v>
+        <v>3565</v>
       </c>
       <c r="J63" s="25" t="s">
-        <v>3707</v>
+        <v>3566</v>
       </c>
       <c r="K63" t="s">
-        <v>3556</v>
+        <v>3567</v>
       </c>
       <c r="L63" s="1" t="s">
-        <v>3557</v>
+        <v>3568</v>
       </c>
       <c r="M63" t="s">
-        <v>3558</v>
+        <v>3569</v>
       </c>
       <c r="N63" t="s">
-        <v>3559</v>
+        <v>3570</v>
       </c>
       <c r="P63" s="1" t="s">
-        <v>3560</v>
+        <v>3571</v>
       </c>
       <c r="Q63" s="1" t="s">
-        <v>3561</v>
+        <v>3572</v>
       </c>
       <c r="R63" s="1" t="s">
-        <v>3562</v>
+        <v>3573</v>
       </c>
       <c r="S63" s="1" t="s">
-        <v>3563</v>
+        <v>3574</v>
       </c>
       <c r="T63" s="1" t="s">
-        <v>3564</v>
+        <v>3575</v>
       </c>
       <c r="U63" s="1" t="s">
-        <v>3565</v>
+        <v>3576</v>
       </c>
       <c r="V63" s="1" t="s">
-        <v>3566</v>
+        <v>3577</v>
       </c>
       <c r="W63" s="1" t="s">
-        <v>3567</v>
+        <v>3578</v>
       </c>
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>3568</v>
+        <v>3579</v>
       </c>
       <c r="C64" t="s">
-        <v>3569</v>
+        <v>3580</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>3552</v>
+        <v>3562</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>3553</v>
+        <v>3563</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>3570</v>
+        <v>3581</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>3571</v>
+        <v>3582</v>
       </c>
       <c r="J64" t="s">
-        <v>3572</v>
+        <v>3583</v>
       </c>
       <c r="K64" t="s">
-        <v>3573</v>
+        <v>3584</v>
       </c>
       <c r="L64" s="1" t="s">
-        <v>3574</v>
+        <v>3585</v>
       </c>
       <c r="M64" t="s">
-        <v>3575</v>
+        <v>3586</v>
       </c>
       <c r="N64" t="s">
-        <v>3576</v>
+        <v>3587</v>
       </c>
       <c r="P64" s="1" t="s">
-        <v>3577</v>
+        <v>3588</v>
       </c>
       <c r="Q64" s="1" t="s">
-        <v>3578</v>
+        <v>3589</v>
       </c>
       <c r="R64" s="1" t="s">
-        <v>3579</v>
+        <v>3590</v>
       </c>
       <c r="S64" s="1" t="s">
-        <v>3580</v>
+        <v>3591</v>
       </c>
       <c r="T64" s="1" t="s">
-        <v>3581</v>
+        <v>3592</v>
       </c>
       <c r="U64" s="1" t="s">
-        <v>3582</v>
+        <v>3593</v>
       </c>
       <c r="V64" s="1" t="s">
-        <v>3583</v>
+        <v>3594</v>
       </c>
       <c r="W64" s="1" t="s">
-        <v>3584</v>
+        <v>3595</v>
       </c>
     </row>
     <row r="65" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>3585</v>
+        <v>3596</v>
       </c>
       <c r="C65" t="s">
-        <v>3586</v>
+        <v>3597</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>3552</v>
+        <v>3562</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>3553</v>
+        <v>3563</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>3587</v>
+        <v>3598</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>3588</v>
+        <v>3599</v>
       </c>
       <c r="J65" t="s">
-        <v>3589</v>
+        <v>3600</v>
       </c>
       <c r="K65" t="s">
-        <v>3590</v>
+        <v>3601</v>
       </c>
       <c r="L65" s="1" t="s">
-        <v>3591</v>
+        <v>3602</v>
       </c>
       <c r="M65" t="s">
-        <v>3592</v>
+        <v>3603</v>
       </c>
       <c r="N65" t="s">
-        <v>3593</v>
+        <v>3604</v>
       </c>
       <c r="P65" s="1" t="s">
-        <v>3594</v>
+        <v>3605</v>
       </c>
       <c r="Q65" s="1" t="s">
-        <v>3595</v>
+        <v>3606</v>
       </c>
       <c r="R65" s="1" t="s">
-        <v>3596</v>
+        <v>3607</v>
       </c>
       <c r="S65" s="1" t="s">
-        <v>3597</v>
+        <v>3608</v>
       </c>
       <c r="T65" s="1" t="s">
-        <v>3598</v>
+        <v>3609</v>
       </c>
       <c r="U65" s="1" t="s">
-        <v>3599</v>
+        <v>3610</v>
       </c>
       <c r="V65" s="1" t="s">
-        <v>3600</v>
+        <v>3611</v>
       </c>
       <c r="W65" s="1" t="s">
-        <v>3601</v>
+        <v>3612</v>
       </c>
     </row>
     <row r="66" spans="1:23" x14ac:dyDescent="0.2">
@@ -27484,13 +27544,13 @@
         <v>2963</v>
       </c>
       <c r="C66" t="s">
-        <v>3602</v>
+        <v>3613</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>3552</v>
+        <v>3562</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>3553</v>
+        <v>3563</v>
       </c>
       <c r="H66" s="1" t="s">
         <v>2964</v>
@@ -27499,146 +27559,146 @@
         <v>2965</v>
       </c>
       <c r="J66" t="s">
-        <v>3603</v>
+        <v>3614</v>
       </c>
       <c r="K66" t="s">
-        <v>3604</v>
+        <v>3615</v>
       </c>
       <c r="L66" s="1" t="s">
-        <v>3605</v>
+        <v>3616</v>
       </c>
       <c r="M66" t="s">
-        <v>3606</v>
+        <v>3617</v>
       </c>
       <c r="N66" t="s">
-        <v>3607</v>
+        <v>3618</v>
       </c>
       <c r="P66" s="1" t="s">
         <v>2967</v>
       </c>
       <c r="Q66" s="1" t="s">
-        <v>3608</v>
+        <v>3619</v>
       </c>
       <c r="R66" s="1" t="s">
-        <v>3609</v>
+        <v>3620</v>
       </c>
       <c r="S66" s="1" t="s">
-        <v>3610</v>
+        <v>3621</v>
       </c>
       <c r="T66" s="1" t="s">
-        <v>3611</v>
+        <v>3622</v>
       </c>
       <c r="U66" s="1" t="s">
-        <v>3612</v>
+        <v>3623</v>
       </c>
       <c r="V66" s="1" t="s">
-        <v>3613</v>
+        <v>3624</v>
       </c>
       <c r="W66" s="1" t="s">
-        <v>3614</v>
+        <v>3625</v>
       </c>
     </row>
     <row r="67" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>3615</v>
+        <v>3626</v>
       </c>
       <c r="C67" t="s">
-        <v>3616</v>
+        <v>3627</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>3552</v>
+        <v>3562</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>3553</v>
+        <v>3563</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>3617</v>
+        <v>3628</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>3618</v>
+        <v>3629</v>
       </c>
       <c r="J67" t="s">
-        <v>3619</v>
+        <v>3630</v>
       </c>
       <c r="K67" s="24" t="s">
-        <v>3620</v>
+        <v>3631</v>
       </c>
       <c r="L67" s="1" t="s">
-        <v>3621</v>
+        <v>3632</v>
       </c>
       <c r="M67" t="s">
-        <v>3622</v>
+        <v>3633</v>
       </c>
       <c r="N67" t="s">
-        <v>3623</v>
+        <v>3634</v>
       </c>
       <c r="P67" s="1" t="s">
-        <v>3624</v>
+        <v>3635</v>
       </c>
       <c r="Q67" s="1" t="s">
-        <v>3625</v>
+        <v>3636</v>
       </c>
       <c r="R67" s="1" t="s">
-        <v>3626</v>
+        <v>3637</v>
       </c>
       <c r="S67" s="1" t="s">
-        <v>3627</v>
+        <v>3638</v>
       </c>
       <c r="T67" s="1" t="s">
-        <v>3628</v>
+        <v>3639</v>
       </c>
       <c r="U67" s="1" t="s">
-        <v>3629</v>
+        <v>3640</v>
       </c>
       <c r="V67" s="1" t="s">
-        <v>3630</v>
+        <v>3641</v>
       </c>
       <c r="W67" s="1" t="s">
-        <v>3377</v>
+        <v>3387</v>
       </c>
     </row>
     <row r="68" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>3402</v>
+        <v>3412</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>3552</v>
+        <v>3562</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>3631</v>
+        <v>3642</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>3403</v>
+        <v>3413</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>3404</v>
+        <v>3414</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>3632</v>
+        <v>3643</v>
       </c>
       <c r="P68" s="1" t="s">
-        <v>3633</v>
+        <v>3644</v>
       </c>
       <c r="Q68" s="1" t="s">
-        <v>3634</v>
+        <v>3645</v>
       </c>
       <c r="R68" s="1" t="s">
-        <v>3635</v>
+        <v>3646</v>
       </c>
       <c r="S68" s="1" t="s">
-        <v>3636</v>
+        <v>3647</v>
       </c>
       <c r="T68" s="1" t="s">
-        <v>3637</v>
+        <v>3648</v>
       </c>
       <c r="U68" s="1" t="s">
-        <v>3638</v>
+        <v>3649</v>
       </c>
       <c r="V68" s="1" t="s">
-        <v>3639</v>
+        <v>3650</v>
       </c>
       <c r="W68" s="1" t="s">
-        <v>3412</v>
+        <v>3422</v>
       </c>
     </row>
   </sheetData>
@@ -27693,7 +27753,7 @@
         <v>9</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>3640</v>
+        <v>3651</v>
       </c>
       <c r="L1" s="5" t="s">
         <v>10</v>
@@ -27705,18 +27765,18 @@
         <v>12</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>3641</v>
+        <v>3652</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>3642</v>
+        <v>3653</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>3643</v>
+        <v>3654</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>3644</v>
+        <v>3655</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4" t="s">
@@ -27726,40 +27786,40 @@
         <v>2244</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>3645</v>
+        <v>3656</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>3646</v>
+        <v>3657</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>3647</v>
+        <v>3658</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>3648</v>
+        <v>3659</v>
       </c>
       <c r="K2" s="4"/>
       <c r="L2" s="4" t="s">
-        <v>3649</v>
+        <v>3660</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>3650</v>
+        <v>3661</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>3651</v>
+        <v>3662</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>3652</v>
+        <v>3663</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>3653</v>
+        <v>3664</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>3654</v>
+        <v>3665</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>3655</v>
+        <v>3666</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
@@ -27769,40 +27829,40 @@
         <v>2244</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>3656</v>
+        <v>3667</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>3657</v>
+        <v>3668</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>3658</v>
+        <v>3669</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>3659</v>
+        <v>3670</v>
       </c>
       <c r="K3" s="4"/>
       <c r="L3" s="4" t="s">
-        <v>3660</v>
+        <v>3671</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>3661</v>
+        <v>3672</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>3662</v>
+        <v>3673</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>3663</v>
+        <v>3674</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>3664</v>
+        <v>3675</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>3665</v>
+        <v>3676</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>3666</v>
+        <v>3677</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4" t="s">
@@ -27812,40 +27872,40 @@
         <v>2244</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>3667</v>
+        <v>3678</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>3668</v>
+        <v>3679</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>3669</v>
+        <v>3680</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>3670</v>
+        <v>3681</v>
       </c>
       <c r="K4" s="4"/>
       <c r="L4" s="4" t="s">
-        <v>3671</v>
+        <v>3682</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>3672</v>
+        <v>3683</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>3673</v>
+        <v>3684</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>3674</v>
+        <v>3685</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>3675</v>
+        <v>3686</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>3676</v>
+        <v>3687</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>3677</v>
+        <v>3688</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4" t="s">
@@ -27855,40 +27915,40 @@
         <v>2244</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>3678</v>
+        <v>3689</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>3679</v>
+        <v>3690</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>3680</v>
+        <v>3691</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>3681</v>
+        <v>3692</v>
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4" t="s">
-        <v>3682</v>
+        <v>3693</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>3683</v>
+        <v>3694</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>3684</v>
+        <v>3695</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>3685</v>
+        <v>3696</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>3686</v>
+        <v>3697</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>3687</v>
+        <v>3698</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>3688</v>
+        <v>3699</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4" t="s">
@@ -27898,37 +27958,37 @@
         <v>2244</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>3689</v>
+        <v>3700</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>3690</v>
+        <v>3701</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>3691</v>
+        <v>3702</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>3692</v>
+        <v>3703</v>
       </c>
       <c r="K6" s="4"/>
       <c r="L6" s="4" t="s">
-        <v>3693</v>
+        <v>3704</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>3694</v>
+        <v>3705</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>3695</v>
+        <v>3706</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>3696</v>
+        <v>3707</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>3697</v>
+        <v>3708</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>3698</v>
+        <v>3709</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
@@ -27939,29 +27999,29 @@
         <v>2244</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>3699</v>
+        <v>3710</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>3700</v>
+        <v>3711</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>3701</v>
+        <v>3712</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>3702</v>
+        <v>3713</v>
       </c>
       <c r="K7" s="4"/>
       <c r="L7" s="4" t="s">
-        <v>3703</v>
+        <v>3714</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>3704</v>
+        <v>3715</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>3705</v>
+        <v>3716</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>3706</v>
+        <v>3717</v>
       </c>
     </row>
   </sheetData>

</xml_diff>